<commit_message>
GBDS JULY 2026 | berlyn@gbds
</commit_message>
<xml_diff>
--- a/GBDS JULY FILES 2026/CSR MONTH OF JULY 2026.xlsx
+++ b/GBDS JULY FILES 2026/CSR MONTH OF JULY 2026.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\GBDS JULY FILES 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3FEE021-DC58-4406-975C-B0B8BD65F1E2}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42594E29-CCA8-4A57-996B-0C2D8CBB9B34}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="4" xr2:uid="{67C3A74A-A57E-4AB5-8CD3-31B592A14032}"/>
   </bookViews>
   <sheets>
     <sheet name="CSR | JULY" sheetId="902" r:id="rId1"/>
     <sheet name="(1)" sheetId="1790" r:id="rId2"/>
-    <sheet name="07-01 R1" sheetId="1791" r:id="rId3"/>
+    <sheet name="07-01 R1 NO TRIP" sheetId="1791" r:id="rId3"/>
     <sheet name="07-01 R2" sheetId="1792" r:id="rId4"/>
     <sheet name="07-01 R3" sheetId="1793" r:id="rId5"/>
     <sheet name="(2)" sheetId="1794" r:id="rId6"/>
@@ -39,7 +39,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="5">'(2)'!$A$1:$Z$44</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="9">'(3)'!$A$1:$Z$44</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="13">'(4)'!$A$1:$Z$44</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'07-01 R1'!$A$1:$Z$43</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'07-01 R1 NO TRIP'!$A$1:$Z$43</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'07-01 R2'!$A$1:$V$44</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="4">'07-01 R3'!$A$1:$V$44</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="6">'07-02 R1'!$A$1:$Z$43</definedName>
@@ -68,7 +68,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1374" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1385" uniqueCount="81">
   <si>
     <t>CHECKER STOCK REPORT</t>
   </si>
@@ -290,6 +290,27 @@
   </si>
   <si>
     <t>DATE ___________07/04/2026___________</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>10/12B</t>
+  </si>
+  <si>
+    <t>11/12B</t>
+  </si>
+  <si>
+    <t>1/12B</t>
+  </si>
+  <si>
+    <t>9/4B</t>
+  </si>
+  <si>
+    <t>12/12B</t>
+  </si>
+  <si>
+    <t>3/3B</t>
   </si>
 </sst>
 </file>
@@ -18220,12 +18241,20 @@
     </row>
     <row r="8" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="12"/>
-      <c r="C8" s="77"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
+      <c r="C8" s="77" t="s">
+        <v>74</v>
+      </c>
+      <c r="D8" s="14">
+        <v>1</v>
+      </c>
+      <c r="E8" s="14">
+        <v>1</v>
+      </c>
       <c r="F8" s="14"/>
       <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
+      <c r="H8" s="14" t="s">
+        <v>76</v>
+      </c>
       <c r="I8" s="14"/>
       <c r="J8" s="14"/>
       <c r="K8" s="14"/>
@@ -18236,12 +18265,18 @@
       <c r="P8" s="14"/>
       <c r="Q8" s="14"/>
       <c r="R8" s="14"/>
-      <c r="S8" s="14"/>
+      <c r="S8" s="14">
+        <v>1</v>
+      </c>
       <c r="T8" s="14"/>
       <c r="U8" s="14"/>
       <c r="V8" s="14"/>
-      <c r="W8" s="14"/>
-      <c r="X8" s="59"/>
+      <c r="W8" s="14">
+        <v>5</v>
+      </c>
+      <c r="X8" s="59">
+        <v>1</v>
+      </c>
       <c r="Y8" s="15"/>
     </row>
     <row r="9" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
@@ -18408,12 +18443,20 @@
       <c r="B15" s="21" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="22"/>
-      <c r="D15" s="23"/>
-      <c r="E15" s="23"/>
+      <c r="C15" s="22">
+        <v>1</v>
+      </c>
+      <c r="D15" s="23">
+        <v>1</v>
+      </c>
+      <c r="E15" s="23">
+        <v>1</v>
+      </c>
       <c r="F15" s="23"/>
       <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
+      <c r="H15" s="23">
+        <v>1</v>
+      </c>
       <c r="I15" s="23"/>
       <c r="J15" s="23"/>
       <c r="K15" s="23"/>
@@ -18424,24 +18467,38 @@
       <c r="P15" s="23"/>
       <c r="Q15" s="23"/>
       <c r="R15" s="23"/>
-      <c r="S15" s="23"/>
+      <c r="S15" s="23">
+        <v>1</v>
+      </c>
       <c r="T15" s="23"/>
       <c r="U15" s="23"/>
       <c r="V15" s="23"/>
-      <c r="W15" s="23"/>
-      <c r="X15" s="61"/>
+      <c r="W15" s="23">
+        <v>0</v>
+      </c>
+      <c r="X15" s="61">
+        <v>0</v>
+      </c>
       <c r="Y15" s="24"/>
     </row>
     <row r="16" spans="2:27" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="C16" s="57"/>
-      <c r="D16" s="58"/>
-      <c r="E16" s="27"/>
+      <c r="C16" s="57">
+        <v>0</v>
+      </c>
+      <c r="D16" s="58">
+        <v>0</v>
+      </c>
+      <c r="E16" s="27">
+        <v>0</v>
+      </c>
       <c r="F16" s="27"/>
       <c r="G16" s="28"/>
-      <c r="H16" s="28"/>
+      <c r="H16" s="28" t="s">
+        <v>75</v>
+      </c>
       <c r="I16" s="28"/>
       <c r="J16" s="28"/>
       <c r="K16" s="56"/>
@@ -18452,12 +18509,18 @@
       <c r="P16" s="28"/>
       <c r="Q16" s="28"/>
       <c r="R16" s="28"/>
-      <c r="S16" s="28"/>
+      <c r="S16" s="28">
+        <v>0</v>
+      </c>
       <c r="T16" s="28"/>
       <c r="U16" s="28"/>
       <c r="V16" s="28"/>
-      <c r="W16" s="56"/>
-      <c r="X16" s="62"/>
+      <c r="W16" s="56">
+        <v>5</v>
+      </c>
+      <c r="X16" s="62">
+        <v>1</v>
+      </c>
       <c r="Y16" s="29"/>
     </row>
     <row r="17" spans="2:25" s="5" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -18860,17 +18923,29 @@
       <c r="C24" s="13"/>
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
-      <c r="F24" s="79"/>
+      <c r="F24" s="79" t="s">
+        <v>77</v>
+      </c>
       <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
+      <c r="H24" s="14">
+        <v>55</v>
+      </c>
       <c r="I24" s="14"/>
       <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
+      <c r="K24" s="14">
+        <v>2</v>
+      </c>
+      <c r="L24" s="14">
+        <v>10</v>
+      </c>
+      <c r="M24" s="14">
+        <v>366</v>
+      </c>
       <c r="N24" s="14"/>
       <c r="O24" s="14"/>
-      <c r="P24" s="14"/>
+      <c r="P24" s="14" t="s">
+        <v>78</v>
+      </c>
       <c r="Q24" s="14"/>
       <c r="R24" s="14"/>
       <c r="S24" s="14"/>
@@ -19046,17 +19121,29 @@
       <c r="C31" s="22"/>
       <c r="D31" s="23"/>
       <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
+      <c r="F31" s="23" t="s">
+        <v>77</v>
+      </c>
       <c r="G31" s="23"/>
-      <c r="H31" s="23"/>
+      <c r="H31" s="23">
+        <v>1</v>
+      </c>
       <c r="I31" s="23"/>
       <c r="J31" s="23"/>
-      <c r="K31" s="23"/>
-      <c r="L31" s="23"/>
-      <c r="M31" s="23"/>
+      <c r="K31" s="23">
+        <v>2</v>
+      </c>
+      <c r="L31" s="23">
+        <v>2</v>
+      </c>
+      <c r="M31" s="23">
+        <v>110</v>
+      </c>
       <c r="N31" s="23"/>
       <c r="O31" s="23"/>
-      <c r="P31" s="23"/>
+      <c r="P31" s="23" t="s">
+        <v>78</v>
+      </c>
       <c r="Q31" s="23"/>
       <c r="R31" s="23"/>
       <c r="S31" s="23"/>
@@ -19074,17 +19161,29 @@
       <c r="C32" s="26"/>
       <c r="D32" s="27"/>
       <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
+      <c r="F32" s="27">
+        <v>0</v>
+      </c>
       <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
+      <c r="H32" s="28">
+        <v>54</v>
+      </c>
       <c r="I32" s="28"/>
       <c r="J32" s="28"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="28"/>
+      <c r="K32" s="28">
+        <v>0</v>
+      </c>
+      <c r="L32" s="28">
+        <v>8</v>
+      </c>
+      <c r="M32" s="28">
+        <v>256</v>
+      </c>
       <c r="N32" s="28"/>
       <c r="O32" s="23"/>
-      <c r="P32" s="28"/>
+      <c r="P32" s="28">
+        <v>0</v>
+      </c>
       <c r="Q32" s="28"/>
       <c r="R32" s="28"/>
       <c r="S32" s="28"/>
@@ -19221,21 +19320,39 @@
       <c r="B36" s="52" t="s">
         <v>52</v>
       </c>
-      <c r="C36" s="46"/>
+      <c r="C36" s="46">
+        <v>1</v>
+      </c>
       <c r="D36" s="41"/>
       <c r="E36" s="42"/>
-      <c r="F36" s="42"/>
-      <c r="G36" s="42"/>
-      <c r="H36" s="42"/>
-      <c r="I36" s="42"/>
+      <c r="F36" s="42">
+        <v>316</v>
+      </c>
+      <c r="G36" s="42">
+        <v>1</v>
+      </c>
+      <c r="H36" s="42">
+        <v>5</v>
+      </c>
+      <c r="I36" s="42">
+        <v>3</v>
+      </c>
       <c r="J36" s="42"/>
       <c r="K36" s="42"/>
-      <c r="L36" s="42"/>
+      <c r="L36" s="42">
+        <v>4</v>
+      </c>
       <c r="M36" s="42"/>
       <c r="N36" s="42"/>
-      <c r="O36" s="42"/>
-      <c r="P36" s="42"/>
-      <c r="Q36" s="43"/>
+      <c r="O36" s="42">
+        <v>5</v>
+      </c>
+      <c r="P36" s="42">
+        <v>6</v>
+      </c>
+      <c r="Q36" s="43">
+        <v>9</v>
+      </c>
       <c r="R36" s="72"/>
       <c r="S36" s="44"/>
       <c r="T36" s="44"/>
@@ -19379,21 +19496,39 @@
       <c r="B42" s="45" t="s">
         <v>53</v>
       </c>
-      <c r="C42" s="46"/>
+      <c r="C42" s="46">
+        <v>1</v>
+      </c>
       <c r="D42" s="41"/>
       <c r="E42" s="42"/>
-      <c r="F42" s="42"/>
-      <c r="G42" s="42"/>
-      <c r="H42" s="42"/>
-      <c r="I42" s="42"/>
+      <c r="F42" s="42">
+        <v>316</v>
+      </c>
+      <c r="G42" s="42">
+        <v>1</v>
+      </c>
+      <c r="H42" s="42">
+        <v>5</v>
+      </c>
+      <c r="I42" s="42">
+        <v>3</v>
+      </c>
       <c r="J42" s="42"/>
       <c r="K42" s="42"/>
-      <c r="L42" s="42"/>
+      <c r="L42" s="42">
+        <v>4</v>
+      </c>
       <c r="M42" s="42"/>
       <c r="N42" s="42"/>
-      <c r="O42" s="42"/>
-      <c r="P42" s="42"/>
-      <c r="Q42" s="43"/>
+      <c r="O42" s="42">
+        <v>5</v>
+      </c>
+      <c r="P42" s="42">
+        <v>6</v>
+      </c>
+      <c r="Q42" s="43">
+        <v>9</v>
+      </c>
       <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
@@ -19435,7 +19570,10 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
+      <c r="C44" s="92">
+        <f>10+5+1+54+8+256</f>
+        <v>334</v>
+      </c>
       <c r="D44" s="92"/>
       <c r="E44" s="92"/>
     </row>
@@ -19443,7 +19581,9 @@
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
+      <c r="C45" s="92">
+        <v>12</v>
+      </c>
       <c r="D45" s="92"/>
       <c r="E45" s="92"/>
     </row>
@@ -19844,11 +19984,17 @@
     <row r="8" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="12"/>
       <c r="C8" s="13"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
+      <c r="D8" s="14">
+        <v>2</v>
+      </c>
+      <c r="E8" s="14">
+        <v>2</v>
+      </c>
       <c r="F8" s="14"/>
       <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
+      <c r="H8" s="14">
+        <v>24</v>
+      </c>
       <c r="I8" s="14"/>
       <c r="J8" s="14"/>
       <c r="K8" s="14"/>
@@ -19860,12 +20006,20 @@
       <c r="Q8" s="14"/>
       <c r="R8" s="14"/>
       <c r="S8" s="14"/>
-      <c r="T8" s="14"/>
+      <c r="T8" s="14">
+        <v>2</v>
+      </c>
       <c r="U8" s="14"/>
       <c r="V8" s="14"/>
-      <c r="W8" s="14"/>
-      <c r="X8" s="59"/>
-      <c r="Y8" s="15"/>
+      <c r="W8" s="14">
+        <v>5</v>
+      </c>
+      <c r="X8" s="59">
+        <v>2</v>
+      </c>
+      <c r="Y8" s="15">
+        <v>2</v>
+      </c>
     </row>
     <row r="9" spans="2:27" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="12" t="s">
@@ -20032,11 +20186,17 @@
         <v>25</v>
       </c>
       <c r="C15" s="22"/>
-      <c r="D15" s="23"/>
-      <c r="E15" s="23"/>
+      <c r="D15" s="23">
+        <v>2</v>
+      </c>
+      <c r="E15" s="23">
+        <v>2</v>
+      </c>
       <c r="F15" s="23"/>
       <c r="G15" s="23"/>
-      <c r="H15" s="23"/>
+      <c r="H15" s="23" t="s">
+        <v>76</v>
+      </c>
       <c r="I15" s="23"/>
       <c r="J15" s="23"/>
       <c r="K15" s="23"/>
@@ -20048,23 +20208,37 @@
       <c r="Q15" s="23"/>
       <c r="R15" s="23"/>
       <c r="S15" s="23"/>
-      <c r="T15" s="23"/>
+      <c r="T15" s="23">
+        <v>2</v>
+      </c>
       <c r="U15" s="23"/>
       <c r="V15" s="23"/>
-      <c r="W15" s="23"/>
-      <c r="X15" s="61"/>
-      <c r="Y15" s="24"/>
+      <c r="W15" s="23">
+        <v>0</v>
+      </c>
+      <c r="X15" s="61">
+        <v>2</v>
+      </c>
+      <c r="Y15" s="24">
+        <v>2</v>
+      </c>
     </row>
     <row r="16" spans="2:27" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B16" s="25" t="s">
         <v>26</v>
       </c>
       <c r="C16" s="57"/>
-      <c r="D16" s="58"/>
-      <c r="E16" s="27"/>
+      <c r="D16" s="58">
+        <v>0</v>
+      </c>
+      <c r="E16" s="27">
+        <v>0</v>
+      </c>
       <c r="F16" s="27"/>
       <c r="G16" s="28"/>
-      <c r="H16" s="28"/>
+      <c r="H16" s="28" t="s">
+        <v>79</v>
+      </c>
       <c r="I16" s="28"/>
       <c r="J16" s="28"/>
       <c r="K16" s="56"/>
@@ -20076,12 +20250,20 @@
       <c r="Q16" s="28"/>
       <c r="R16" s="28"/>
       <c r="S16" s="28"/>
-      <c r="T16" s="28"/>
+      <c r="T16" s="28">
+        <v>0</v>
+      </c>
       <c r="U16" s="28"/>
       <c r="V16" s="28"/>
-      <c r="W16" s="56"/>
-      <c r="X16" s="62"/>
-      <c r="Y16" s="29"/>
+      <c r="W16" s="56">
+        <v>5</v>
+      </c>
+      <c r="X16" s="62">
+        <v>0</v>
+      </c>
+      <c r="Y16" s="29">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" spans="2:25" s="5" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="30"/>
@@ -20483,17 +20665,29 @@
       <c r="C24" s="13"/>
       <c r="D24" s="14"/>
       <c r="E24" s="14"/>
-      <c r="F24" s="14"/>
+      <c r="F24" s="14">
+        <v>2</v>
+      </c>
       <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
+      <c r="H24" s="14">
+        <v>55</v>
+      </c>
       <c r="I24" s="14"/>
       <c r="J24" s="14"/>
-      <c r="K24" s="14"/>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
+      <c r="K24" s="14">
+        <v>2</v>
+      </c>
+      <c r="L24" s="14">
+        <v>21</v>
+      </c>
+      <c r="M24" s="14">
+        <v>507</v>
+      </c>
       <c r="N24" s="14"/>
       <c r="O24" s="14"/>
-      <c r="P24" s="14"/>
+      <c r="P24" s="14" t="s">
+        <v>80</v>
+      </c>
       <c r="Q24" s="14"/>
       <c r="R24" s="14"/>
       <c r="S24" s="14"/>
@@ -20669,17 +20863,29 @@
       <c r="C31" s="22"/>
       <c r="D31" s="23"/>
       <c r="E31" s="23"/>
-      <c r="F31" s="23"/>
+      <c r="F31" s="23">
+        <v>2</v>
+      </c>
       <c r="G31" s="23"/>
-      <c r="H31" s="23"/>
+      <c r="H31" s="23">
+        <v>55</v>
+      </c>
       <c r="I31" s="23"/>
       <c r="J31" s="23"/>
-      <c r="K31" s="23"/>
-      <c r="L31" s="23"/>
-      <c r="M31" s="23"/>
+      <c r="K31" s="23">
+        <v>2</v>
+      </c>
+      <c r="L31" s="23">
+        <v>19</v>
+      </c>
+      <c r="M31" s="23">
+        <v>129</v>
+      </c>
       <c r="N31" s="23"/>
       <c r="O31" s="23"/>
-      <c r="P31" s="23"/>
+      <c r="P31" s="23" t="s">
+        <v>80</v>
+      </c>
       <c r="Q31" s="23"/>
       <c r="R31" s="23"/>
       <c r="S31" s="23"/>
@@ -20697,17 +20903,29 @@
       <c r="C32" s="26"/>
       <c r="D32" s="27"/>
       <c r="E32" s="27"/>
-      <c r="F32" s="27"/>
+      <c r="F32" s="27">
+        <v>0</v>
+      </c>
       <c r="G32" s="28"/>
-      <c r="H32" s="28"/>
+      <c r="H32" s="28">
+        <v>0</v>
+      </c>
       <c r="I32" s="28"/>
       <c r="J32" s="28"/>
-      <c r="K32" s="28"/>
-      <c r="L32" s="28"/>
-      <c r="M32" s="28"/>
+      <c r="K32" s="28">
+        <v>0</v>
+      </c>
+      <c r="L32" s="28">
+        <v>2</v>
+      </c>
+      <c r="M32" s="28">
+        <v>378</v>
+      </c>
       <c r="N32" s="28"/>
       <c r="O32" s="23"/>
-      <c r="P32" s="28"/>
+      <c r="P32" s="28">
+        <v>0</v>
+      </c>
       <c r="Q32" s="28"/>
       <c r="R32" s="28"/>
       <c r="S32" s="28"/>
@@ -20847,18 +21065,34 @@
       <c r="C36" s="46"/>
       <c r="D36" s="41"/>
       <c r="E36" s="42"/>
-      <c r="F36" s="42"/>
-      <c r="G36" s="42"/>
-      <c r="H36" s="42"/>
+      <c r="F36" s="42">
+        <v>502</v>
+      </c>
+      <c r="G36" s="42">
+        <v>8</v>
+      </c>
+      <c r="H36" s="42">
+        <v>1</v>
+      </c>
       <c r="I36" s="42"/>
       <c r="J36" s="42"/>
-      <c r="K36" s="42"/>
-      <c r="L36" s="42"/>
+      <c r="K36" s="42">
+        <v>2</v>
+      </c>
+      <c r="L36" s="42">
+        <v>4</v>
+      </c>
       <c r="M36" s="42"/>
       <c r="N36" s="42"/>
-      <c r="O36" s="42"/>
-      <c r="P36" s="42"/>
-      <c r="Q36" s="43"/>
+      <c r="O36" s="42">
+        <v>9</v>
+      </c>
+      <c r="P36" s="42">
+        <v>4</v>
+      </c>
+      <c r="Q36" s="43">
+        <v>1</v>
+      </c>
       <c r="R36" s="72"/>
       <c r="S36" s="44"/>
       <c r="T36" s="44"/>
@@ -21005,18 +21239,34 @@
       <c r="C42" s="46"/>
       <c r="D42" s="41"/>
       <c r="E42" s="42"/>
-      <c r="F42" s="42"/>
-      <c r="G42" s="42"/>
-      <c r="H42" s="42"/>
+      <c r="F42" s="42">
+        <v>502</v>
+      </c>
+      <c r="G42" s="42">
+        <v>8</v>
+      </c>
+      <c r="H42" s="42">
+        <v>1</v>
+      </c>
       <c r="I42" s="42"/>
       <c r="J42" s="42"/>
-      <c r="K42" s="42"/>
-      <c r="L42" s="42"/>
+      <c r="K42" s="42">
+        <v>2</v>
+      </c>
+      <c r="L42" s="42">
+        <v>4</v>
+      </c>
       <c r="M42" s="42"/>
       <c r="N42" s="42"/>
-      <c r="O42" s="42"/>
-      <c r="P42" s="42"/>
-      <c r="Q42" s="43"/>
+      <c r="O42" s="42">
+        <v>9</v>
+      </c>
+      <c r="P42" s="42">
+        <v>4</v>
+      </c>
+      <c r="Q42" s="43">
+        <v>1</v>
+      </c>
       <c r="R42" s="84" t="s">
         <v>54</v>
       </c>
@@ -21058,7 +21308,10 @@
       <c r="B44" s="76" t="s">
         <v>68</v>
       </c>
-      <c r="C44" s="92"/>
+      <c r="C44" s="92">
+        <f>12+5+2+378</f>
+        <v>397</v>
+      </c>
       <c r="D44" s="92"/>
       <c r="E44" s="92"/>
     </row>
@@ -21066,7 +21319,9 @@
       <c r="B45" s="76" t="s">
         <v>69</v>
       </c>
-      <c r="C45" s="92"/>
+      <c r="C45" s="92">
+        <v>12</v>
+      </c>
       <c r="D45" s="92"/>
       <c r="E45" s="92"/>
     </row>

</xml_diff>